<commit_message>
feat: Incluir tipos contabilidad ifrs4 local y corporativo
</commit_message>
<xml_diff>
--- a/prototipo_pcr/inputs/nomenclatura.xlsx
+++ b/prototipo_pcr/inputs/nomenclatura.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\samuarta\Proyectos\prototipo-pcr\prototipo_pcr\inputs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2EB65200-B037-47B7-85F3-C51DD2FACE12}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2D2FC32F-F030-4A50-A018-18D5F9CA385E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="1" xr2:uid="{B6BBB8B8-7677-D84C-AD85-43B73374E2C3}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{B6BBB8B8-7677-D84C-AD85-43B73374E2C3}"/>
   </bookViews>
   <sheets>
     <sheet name="V1" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="837" uniqueCount="382">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="844" uniqueCount="385">
   <si>
     <t>Campo</t>
   </si>
@@ -45,9 +45,6 @@
     <t>tipo_contabilidad</t>
   </si>
   <si>
-    <t>ifrs4</t>
-  </si>
-  <si>
     <t>ifrs17_local</t>
   </si>
   <si>
@@ -1183,6 +1180,18 @@
   </si>
   <si>
     <t>NO</t>
+  </si>
+  <si>
+    <t>ifrs4_local</t>
+  </si>
+  <si>
+    <t>ifrs4_corporativo</t>
+  </si>
+  <si>
+    <t>NIIF4C</t>
+  </si>
+  <si>
+    <t>NIIF4L</t>
   </si>
 </sst>
 </file>
@@ -1323,7 +1332,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="34">
+  <cellXfs count="37">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
@@ -1380,6 +1389,11 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1714,7 +1728,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2FA1C9BF-152D-454C-B2E4-5B164FCAC037}">
-  <dimension ref="A1:E69"/>
+  <dimension ref="A1:E70"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="1" width="27" bestFit="1" customWidth="1"/>
@@ -1729,75 +1743,75 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A2" s="3" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="C2" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="D2" s="3"/>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A3" s="3" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B3" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="C3" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="D3" s="3"/>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A4" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="B4" t="s">
+        <v>114</v>
+      </c>
+      <c r="C4" t="s">
         <v>8</v>
-      </c>
-      <c r="B4" t="s">
-        <v>115</v>
-      </c>
-      <c r="C4" t="s">
-        <v>9</v>
       </c>
       <c r="D4" s="3"/>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A5" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="B5" t="s">
+        <v>115</v>
+      </c>
+      <c r="C5" t="s">
         <v>8</v>
-      </c>
-      <c r="B5" t="s">
-        <v>116</v>
-      </c>
-      <c r="C5" t="s">
-        <v>9</v>
       </c>
       <c r="D5" s="3"/>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A6" s="4" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="D6" s="4"/>
       <c r="E6" s="5"/>
@@ -1807,10 +1821,10 @@
         <v>1</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>2</v>
+        <v>381</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>5</v>
+        <v>384</v>
       </c>
       <c r="D7" s="6"/>
       <c r="E7" s="6"/>
@@ -1820,808 +1834,821 @@
         <v>1</v>
       </c>
       <c r="B8" t="s">
+        <v>382</v>
+      </c>
+      <c r="C8" t="s">
+        <v>383</v>
+      </c>
+      <c r="D8" s="36"/>
+      <c r="E8" s="36"/>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A9" t="s">
+        <v>1</v>
+      </c>
+      <c r="B9" t="s">
+        <v>2</v>
+      </c>
+      <c r="C9" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A10" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="B10" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="C8" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.4">
-      <c r="A9" s="5" t="s">
-        <v>1</v>
-      </c>
-      <c r="B9" s="5" t="s">
-        <v>4</v>
-      </c>
-      <c r="C9" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="D9" s="5"/>
-      <c r="E9" s="5"/>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.4">
-      <c r="A10" s="6" t="s">
+      <c r="C10" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="D10" s="5"/>
+      <c r="E10" s="5"/>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A11" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="B11" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="B10" s="6" t="s">
+      <c r="C11" s="7" t="s">
+        <v>52</v>
+      </c>
+      <c r="D11" s="7" t="s">
+        <v>127</v>
+      </c>
+      <c r="E11" s="6" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A12" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B12" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="C10" s="7" t="s">
+      <c r="C12" s="8" t="s">
         <v>53</v>
       </c>
-      <c r="D10" s="7" t="s">
+      <c r="D12" s="8" t="s">
         <v>128</v>
       </c>
-      <c r="E10" s="6" t="s">
-        <v>147</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.4">
-      <c r="A11" s="5" t="s">
-        <v>10</v>
-      </c>
-      <c r="B11" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="C11" s="8" t="s">
+      <c r="E12" s="6" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A13" s="6" t="s">
         <v>54</v>
       </c>
-      <c r="D11" s="8" t="s">
-        <v>129</v>
-      </c>
-      <c r="E11" s="6" t="s">
-        <v>147</v>
-      </c>
-    </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.4">
-      <c r="A12" s="6" t="s">
-        <v>55</v>
-      </c>
-      <c r="B12" s="6" t="s">
-        <v>45</v>
-      </c>
-      <c r="C12" s="6" t="s">
-        <v>27</v>
-      </c>
-      <c r="D12" s="6" t="s">
+      <c r="B13" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="C13" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="D13" s="6" t="s">
+        <v>130</v>
+      </c>
+      <c r="E13" s="6"/>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A14" s="5" t="s">
+        <v>54</v>
+      </c>
+      <c r="B14" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="C14" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="D14" s="5" t="s">
         <v>131</v>
       </c>
-      <c r="E12" s="6"/>
-    </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.4">
-      <c r="A13" s="5" t="s">
-        <v>55</v>
-      </c>
-      <c r="B13" s="5" t="s">
-        <v>47</v>
-      </c>
-      <c r="C13" s="5" t="s">
-        <v>30</v>
-      </c>
-      <c r="D13" s="5" t="s">
-        <v>132</v>
-      </c>
-      <c r="E13" s="5"/>
-    </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.4">
-      <c r="A14" s="6" t="s">
-        <v>73</v>
-      </c>
-      <c r="B14" s="6" t="s">
-        <v>57</v>
-      </c>
-      <c r="C14" s="6" t="s">
-        <v>27</v>
-      </c>
-      <c r="D14" s="6"/>
-      <c r="E14" s="6"/>
+      <c r="E14" s="5"/>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.4">
-      <c r="A15" t="s">
-        <v>73</v>
-      </c>
-      <c r="B15" t="s">
-        <v>58</v>
-      </c>
-      <c r="C15" t="s">
+      <c r="A15" s="6" t="s">
+        <v>72</v>
+      </c>
+      <c r="B15" s="6" t="s">
         <v>56</v>
       </c>
+      <c r="C15" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="D15" s="6"/>
+      <c r="E15" s="6"/>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A16" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B16" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="C16" t="s">
-        <v>29</v>
+        <v>55</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A17" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B17" t="s">
+        <v>58</v>
+      </c>
+      <c r="C17" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A18" t="s">
+        <v>72</v>
+      </c>
+      <c r="B18" t="s">
+        <v>59</v>
+      </c>
+      <c r="C18" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A19" s="9" t="s">
+        <v>72</v>
+      </c>
+      <c r="B19" s="9" t="s">
+        <v>155</v>
+      </c>
+      <c r="C19" s="9" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A20" s="5" t="s">
+        <v>72</v>
+      </c>
+      <c r="B20" s="5" t="s">
         <v>60</v>
       </c>
-      <c r="C17" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.4">
-      <c r="A18" s="9" t="s">
-        <v>73</v>
-      </c>
-      <c r="B18" s="9" t="s">
-        <v>156</v>
-      </c>
-      <c r="C18" s="9" t="s">
-        <v>159</v>
-      </c>
-    </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.4">
-      <c r="A19" s="5" t="s">
-        <v>73</v>
-      </c>
-      <c r="B19" s="5" t="s">
-        <v>61</v>
-      </c>
-      <c r="C19" s="5" t="s">
-        <v>30</v>
-      </c>
-      <c r="D19" s="5"/>
-      <c r="E19" s="5"/>
-    </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.4">
-      <c r="A20" s="6" t="s">
+      <c r="C20" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="D20" s="5"/>
+      <c r="E20" s="5"/>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A21" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="B21" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="B20" s="6" t="s">
+      <c r="C21" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="D21" s="6"/>
+      <c r="E21" s="6"/>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A22" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="B22" s="9" t="s">
         <v>14</v>
       </c>
-      <c r="C20" s="6" t="s">
+      <c r="C22" s="9" t="s">
         <v>37</v>
       </c>
-      <c r="D20" s="6"/>
-      <c r="E20" s="6"/>
-    </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.4">
-      <c r="A21" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="B21" s="9" t="s">
-        <v>15</v>
-      </c>
-      <c r="C21" s="9" t="s">
-        <v>38</v>
-      </c>
-      <c r="D21" s="9"/>
-      <c r="E21" s="9" t="s">
-        <v>148</v>
-      </c>
-    </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.4">
-      <c r="A22" t="s">
-        <v>13</v>
-      </c>
-      <c r="B22" t="s">
-        <v>16</v>
-      </c>
-      <c r="C22" t="s">
-        <v>39</v>
+      <c r="D22" s="9"/>
+      <c r="E22" s="9" t="s">
+        <v>147</v>
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A23" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B23" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="C23" t="s">
-        <v>28</v>
+        <v>38</v>
       </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A24" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B24" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="C24" t="s">
-        <v>40</v>
-      </c>
-      <c r="D24" t="s">
-        <v>133</v>
+        <v>27</v>
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A25" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B25" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="C25" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="D25" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A26" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B26" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="C26" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="D26" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A27" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B27" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="C27" t="s">
+        <v>41</v>
+      </c>
+      <c r="D27" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A28" t="s">
+        <v>12</v>
+      </c>
+      <c r="B28" t="s">
+        <v>20</v>
+      </c>
+      <c r="C28" t="s">
+        <v>42</v>
+      </c>
+      <c r="D28" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A29" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="B29" s="9" t="s">
+        <v>148</v>
+      </c>
+      <c r="C29" s="9" t="s">
         <v>43</v>
       </c>
-      <c r="D27" t="s">
-        <v>136</v>
-      </c>
-    </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.4">
-      <c r="A28" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="B28" s="9" t="s">
+      <c r="D29" s="9"/>
+      <c r="E29" s="9" t="s">
         <v>149</v>
-      </c>
-      <c r="C28" s="9" t="s">
-        <v>44</v>
-      </c>
-      <c r="D28" s="9"/>
-      <c r="E28" s="9" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.4">
-      <c r="A29" t="s">
-        <v>13</v>
-      </c>
-      <c r="B29" t="s">
-        <v>23</v>
-      </c>
-      <c r="C29" t="s">
-        <v>34</v>
       </c>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A30" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B30" t="s">
+        <v>22</v>
+      </c>
+      <c r="C30" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A31" t="s">
+        <v>12</v>
+      </c>
+      <c r="B31" t="s">
+        <v>23</v>
+      </c>
+      <c r="C31" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A32" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="B32" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="C30" t="s">
+      <c r="C32" s="5" t="s">
         <v>35</v>
       </c>
-    </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.4">
-      <c r="A31" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="B31" s="5" t="s">
-        <v>25</v>
-      </c>
-      <c r="C31" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="D31" s="5" t="s">
+      <c r="D32" s="5" t="s">
+        <v>136</v>
+      </c>
+      <c r="E32" s="5"/>
+    </row>
+    <row r="33" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A33" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="B33" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="C33" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="D33" s="6" t="s">
         <v>137</v>
       </c>
-      <c r="E31" s="5"/>
-    </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.4">
-      <c r="A32" s="6" t="s">
-        <v>48</v>
-      </c>
-      <c r="B32" s="6" t="s">
+      <c r="E33" s="6"/>
+    </row>
+    <row r="34" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A34" t="s">
+        <v>47</v>
+      </c>
+      <c r="B34" t="s">
         <v>49</v>
       </c>
-      <c r="C32" s="6" t="s">
+      <c r="C34" t="s">
         <v>51</v>
       </c>
-      <c r="D32" s="6" t="s">
+      <c r="D34" t="s">
         <v>138</v>
       </c>
-      <c r="E32" s="6"/>
-    </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.4">
-      <c r="A33" t="s">
-        <v>48</v>
-      </c>
-      <c r="B33" t="s">
-        <v>50</v>
-      </c>
-      <c r="C33" t="s">
-        <v>52</v>
-      </c>
-      <c r="D33" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.4">
-      <c r="A34" s="5" t="s">
-        <v>48</v>
-      </c>
-      <c r="B34" s="5" t="s">
-        <v>25</v>
-      </c>
-      <c r="C34" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="D34" s="5" t="s">
-        <v>137</v>
-      </c>
-      <c r="E34" s="5"/>
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.4">
-      <c r="A35" s="6" t="s">
-        <v>74</v>
-      </c>
-      <c r="B35" s="6" t="s">
-        <v>46</v>
-      </c>
-      <c r="C35" s="6" t="s">
-        <v>27</v>
-      </c>
-      <c r="D35" s="6" t="s">
-        <v>131</v>
-      </c>
-      <c r="E35" s="6"/>
+      <c r="A35" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="B35" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="C35" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="D35" s="5" t="s">
+        <v>136</v>
+      </c>
+      <c r="E35" s="5"/>
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.4">
-      <c r="A36" t="s">
-        <v>74</v>
-      </c>
-      <c r="B36" t="s">
-        <v>62</v>
-      </c>
-      <c r="C36" t="s">
+      <c r="A36" s="6" t="s">
+        <v>73</v>
+      </c>
+      <c r="B36" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="C36" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="D36" t="s">
-        <v>140</v>
-      </c>
+      <c r="D36" s="6" t="s">
+        <v>130</v>
+      </c>
+      <c r="E36" s="6"/>
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A37" t="s">
+        <v>73</v>
+      </c>
+      <c r="B37" t="s">
+        <v>61</v>
+      </c>
+      <c r="C37" t="s">
+        <v>25</v>
+      </c>
+      <c r="D37" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="38" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A38" t="s">
+        <v>73</v>
+      </c>
+      <c r="B38" t="s">
+        <v>62</v>
+      </c>
+      <c r="C38" t="s">
+        <v>64</v>
+      </c>
+      <c r="D38" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="39" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A39" s="5" t="s">
+        <v>73</v>
+      </c>
+      <c r="B39" s="5" t="s">
+        <v>63</v>
+      </c>
+      <c r="C39" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="D39" s="5" t="s">
+        <v>141</v>
+      </c>
+      <c r="E39" s="5"/>
+    </row>
+    <row r="40" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A40" s="6" t="s">
+        <v>65</v>
+      </c>
+      <c r="B40" s="6" t="s">
+        <v>66</v>
+      </c>
+      <c r="C40" s="6" t="s">
+        <v>67</v>
+      </c>
+      <c r="D40" s="6" t="s">
+        <v>142</v>
+      </c>
+      <c r="E40" s="6"/>
+    </row>
+    <row r="41" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A41" t="s">
+        <v>65</v>
+      </c>
+      <c r="B41" t="s">
+        <v>68</v>
+      </c>
+      <c r="C41" t="s">
+        <v>69</v>
+      </c>
+      <c r="D41" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="42" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A42" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="B42" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="C42" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="D42" s="5" t="s">
+        <v>136</v>
+      </c>
+      <c r="E42" s="5"/>
+    </row>
+    <row r="43" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A43" s="6" t="s">
         <v>74</v>
       </c>
-      <c r="B37" t="s">
-        <v>63</v>
-      </c>
-      <c r="C37" t="s">
-        <v>65</v>
-      </c>
-      <c r="D37" t="s">
-        <v>141</v>
-      </c>
-    </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.4">
-      <c r="A38" s="5" t="s">
+      <c r="B43" s="6" t="s">
+        <v>75</v>
+      </c>
+      <c r="C43" s="6" t="s">
+        <v>77</v>
+      </c>
+      <c r="D43" s="6" t="s">
+        <v>144</v>
+      </c>
+      <c r="E43" s="6"/>
+    </row>
+    <row r="44" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A44" t="s">
         <v>74</v>
       </c>
-      <c r="B38" s="5" t="s">
-        <v>64</v>
-      </c>
-      <c r="C38" s="5" t="s">
-        <v>30</v>
-      </c>
-      <c r="D38" s="5" t="s">
-        <v>142</v>
-      </c>
-      <c r="E38" s="5"/>
-    </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.4">
-      <c r="A39" s="6" t="s">
-        <v>66</v>
-      </c>
-      <c r="B39" s="6" t="s">
-        <v>67</v>
-      </c>
-      <c r="C39" s="6" t="s">
-        <v>68</v>
-      </c>
-      <c r="D39" s="6" t="s">
-        <v>143</v>
-      </c>
-      <c r="E39" s="6"/>
-    </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.4">
-      <c r="A40" t="s">
-        <v>66</v>
-      </c>
-      <c r="B40" t="s">
-        <v>69</v>
-      </c>
-      <c r="C40" t="s">
+      <c r="B44" t="s">
+        <v>76</v>
+      </c>
+      <c r="C44" t="s">
+        <v>78</v>
+      </c>
+      <c r="D44" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="45" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A45" s="5" t="s">
+        <v>74</v>
+      </c>
+      <c r="B45" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="C45" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="D45" s="5" t="s">
+        <v>136</v>
+      </c>
+      <c r="E45" s="5"/>
+    </row>
+    <row r="46" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A46" s="6" t="s">
         <v>70</v>
       </c>
-      <c r="D40" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.4">
-      <c r="A41" s="5" t="s">
-        <v>66</v>
-      </c>
-      <c r="B41" s="5" t="s">
-        <v>25</v>
-      </c>
-      <c r="C41" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="D41" s="5" t="s">
-        <v>137</v>
-      </c>
-      <c r="E41" s="5"/>
-    </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.4">
-      <c r="A42" s="6" t="s">
-        <v>75</v>
-      </c>
-      <c r="B42" s="6" t="s">
-        <v>76</v>
-      </c>
-      <c r="C42" s="6" t="s">
-        <v>78</v>
-      </c>
-      <c r="D42" s="6" t="s">
-        <v>145</v>
-      </c>
-      <c r="E42" s="6"/>
-    </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.4">
-      <c r="A43" t="s">
-        <v>75</v>
-      </c>
-      <c r="B43" t="s">
-        <v>77</v>
-      </c>
-      <c r="C43" t="s">
+      <c r="B46" s="6" t="s">
         <v>79</v>
       </c>
-      <c r="D43" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.4">
-      <c r="A44" s="5" t="s">
-        <v>75</v>
-      </c>
-      <c r="B44" s="5" t="s">
-        <v>25</v>
-      </c>
-      <c r="C44" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="D44" s="5" t="s">
-        <v>137</v>
-      </c>
-      <c r="E44" s="5"/>
-    </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.4">
-      <c r="A45" s="6" t="s">
-        <v>71</v>
-      </c>
-      <c r="B45" s="6" t="s">
+      <c r="C46" s="6" t="s">
+        <v>79</v>
+      </c>
+      <c r="D46" s="6"/>
+      <c r="E46" s="6"/>
+    </row>
+    <row r="47" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A47" t="s">
+        <v>70</v>
+      </c>
+      <c r="B47" t="s">
         <v>80</v>
       </c>
-      <c r="C45" s="6" t="s">
-        <v>80</v>
-      </c>
-      <c r="D45" s="6"/>
-      <c r="E45" s="6"/>
-    </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.4">
-      <c r="A46" t="s">
-        <v>71</v>
-      </c>
-      <c r="B46" t="s">
-        <v>81</v>
-      </c>
-      <c r="C46" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.4">
-      <c r="A47" s="10" t="s">
-        <v>71</v>
-      </c>
-      <c r="B47" s="10" t="s">
+      <c r="C47" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="48" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A48" s="10" t="s">
+        <v>70</v>
+      </c>
+      <c r="B48" s="10" t="s">
+        <v>150</v>
+      </c>
+      <c r="C48" s="10" t="s">
         <v>151</v>
-      </c>
-      <c r="C47" s="10" t="s">
-        <v>152</v>
-      </c>
-      <c r="D47" s="9"/>
-      <c r="E47" s="10" t="s">
-        <v>153</v>
-      </c>
-    </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.4">
-      <c r="A48" s="9" t="s">
-        <v>71</v>
-      </c>
-      <c r="B48" s="9" t="s">
-        <v>83</v>
-      </c>
-      <c r="C48" s="9" t="s">
-        <v>121</v>
       </c>
       <c r="D48" s="9"/>
       <c r="E48" s="10" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
     </row>
     <row r="49" spans="1:5" x14ac:dyDescent="0.4">
-      <c r="A49" t="s">
-        <v>71</v>
-      </c>
-      <c r="B49" t="s">
-        <v>93</v>
-      </c>
-      <c r="C49" t="s">
-        <v>122</v>
-      </c>
-    </row>
-    <row r="50" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A49" s="9" t="s">
+        <v>70</v>
+      </c>
+      <c r="B49" s="9" t="s">
+        <v>82</v>
+      </c>
+      <c r="C49" s="9" t="s">
+        <v>120</v>
+      </c>
+      <c r="D49" s="9"/>
+      <c r="E49" s="10" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="50" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A50" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B50" t="s">
-        <v>84</v>
+        <v>92</v>
       </c>
       <c r="C50" t="s">
-        <v>98</v>
+        <v>121</v>
       </c>
     </row>
     <row r="51" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A51" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B51" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="C51" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="52" spans="1:5" x14ac:dyDescent="0.4">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="52" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A52" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B52" t="s">
-        <v>91</v>
+        <v>84</v>
       </c>
       <c r="C52" t="s">
-        <v>104</v>
+        <v>98</v>
       </c>
     </row>
     <row r="53" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A53" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B53" t="s">
         <v>90</v>
       </c>
       <c r="C53" t="s">
-        <v>90</v>
+        <v>103</v>
       </c>
     </row>
     <row r="54" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A54" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B54" t="s">
-        <v>82</v>
+        <v>89</v>
       </c>
       <c r="C54" t="s">
-        <v>97</v>
+        <v>89</v>
       </c>
     </row>
     <row r="55" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A55" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B55" t="s">
-        <v>87</v>
+        <v>81</v>
       </c>
       <c r="C55" t="s">
-        <v>101</v>
+        <v>96</v>
       </c>
     </row>
     <row r="56" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A56" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B56" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="C56" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
     </row>
     <row r="57" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A57" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B57" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="C57" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="58" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="58" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A58" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B58" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="C58" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="59" spans="1:5" x14ac:dyDescent="0.4">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="59" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A59" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B59" t="s">
-        <v>92</v>
+        <v>85</v>
       </c>
       <c r="C59" t="s">
-        <v>105</v>
+        <v>99</v>
       </c>
     </row>
     <row r="60" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A60" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B60" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="C60" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
     </row>
     <row r="61" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A61" t="s">
+        <v>70</v>
+      </c>
+      <c r="B61" t="s">
+        <v>93</v>
+      </c>
+      <c r="C61" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="62" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A62" t="s">
+        <v>70</v>
+      </c>
+      <c r="B62" t="s">
+        <v>94</v>
+      </c>
+      <c r="C62" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="63" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A63" s="12" t="s">
+        <v>70</v>
+      </c>
+      <c r="B63" s="12" t="s">
+        <v>4</v>
+      </c>
+      <c r="C63" s="12" t="s">
+        <v>106</v>
+      </c>
+      <c r="D63" s="12"/>
+      <c r="E63" s="12" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="64" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A64" s="10" t="s">
+        <v>70</v>
+      </c>
+      <c r="B64" s="10" t="s">
+        <v>126</v>
+      </c>
+      <c r="C64" s="10" t="s">
+        <v>126</v>
+      </c>
+      <c r="D64" s="10"/>
+      <c r="E64" s="10" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="65" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A65" s="11" t="s">
+        <v>70</v>
+      </c>
+      <c r="B65" s="11" t="s">
+        <v>125</v>
+      </c>
+      <c r="C65" s="11" t="s">
+        <v>124</v>
+      </c>
+      <c r="D65" s="11"/>
+      <c r="E65" s="11" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="66" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A66" s="6" t="s">
         <v>71</v>
       </c>
-      <c r="B61" t="s">
-        <v>95</v>
-      </c>
-      <c r="C61" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="62" spans="1:5" x14ac:dyDescent="0.4">
-      <c r="A62" s="12" t="s">
-        <v>71</v>
-      </c>
-      <c r="B62" s="12" t="s">
-        <v>5</v>
-      </c>
-      <c r="C62" s="12" t="s">
+      <c r="B66" s="6" t="s">
         <v>107</v>
       </c>
-      <c r="D62" s="12"/>
-      <c r="E62" s="12" t="s">
-        <v>157</v>
-      </c>
-    </row>
-    <row r="63" spans="1:5" x14ac:dyDescent="0.4">
-      <c r="A63" s="10" t="s">
-        <v>71</v>
-      </c>
-      <c r="B63" s="10" t="s">
-        <v>127</v>
-      </c>
-      <c r="C63" s="10" t="s">
-        <v>127</v>
-      </c>
-      <c r="D63" s="10"/>
-      <c r="E63" s="10" t="s">
-        <v>158</v>
-      </c>
-    </row>
-    <row r="64" spans="1:5" x14ac:dyDescent="0.4">
-      <c r="A64" s="11" t="s">
-        <v>71</v>
-      </c>
-      <c r="B64" s="11" t="s">
-        <v>126</v>
-      </c>
-      <c r="C64" s="11" t="s">
-        <v>125</v>
-      </c>
-      <c r="D64" s="11"/>
-      <c r="E64" s="11" t="s">
-        <v>155</v>
-      </c>
-    </row>
-    <row r="65" spans="1:5" x14ac:dyDescent="0.4">
-      <c r="A65" s="6" t="s">
-        <v>72</v>
-      </c>
-      <c r="B65" s="6" t="s">
-        <v>108</v>
-      </c>
-      <c r="C65" s="6" t="s">
-        <v>110</v>
-      </c>
-      <c r="D65" s="6"/>
-      <c r="E65" s="6"/>
-    </row>
-    <row r="66" spans="1:5" x14ac:dyDescent="0.4">
-      <c r="A66" t="s">
-        <v>72</v>
-      </c>
-      <c r="B66" t="s">
-        <v>82</v>
-      </c>
-      <c r="C66" t="s">
-        <v>97</v>
-      </c>
+      <c r="C66" s="6" t="s">
+        <v>109</v>
+      </c>
+      <c r="D66" s="6"/>
+      <c r="E66" s="6"/>
     </row>
     <row r="67" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A67" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B67" t="s">
-        <v>22</v>
+        <v>81</v>
       </c>
       <c r="C67" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="68" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A68" t="s">
+        <v>71</v>
+      </c>
+      <c r="B68" t="s">
+        <v>21</v>
+      </c>
+      <c r="C68" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="69" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A69" s="9" t="s">
+        <v>71</v>
+      </c>
+      <c r="B69" s="9" t="s">
+        <v>119</v>
+      </c>
+      <c r="C69" s="9" t="s">
+        <v>30</v>
+      </c>
+      <c r="D69" s="9"/>
+      <c r="E69" s="10" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="70" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A70" t="s">
+        <v>71</v>
+      </c>
+      <c r="B70" t="s">
+        <v>108</v>
+      </c>
+      <c r="C70" t="s">
         <v>32</v>
-      </c>
-    </row>
-    <row r="68" spans="1:5" x14ac:dyDescent="0.4">
-      <c r="A68" s="9" t="s">
-        <v>72</v>
-      </c>
-      <c r="B68" s="9" t="s">
-        <v>120</v>
-      </c>
-      <c r="C68" s="9" t="s">
-        <v>31</v>
-      </c>
-      <c r="D68" s="9"/>
-      <c r="E68" s="10" t="s">
-        <v>124</v>
-      </c>
-    </row>
-    <row r="69" spans="1:5" x14ac:dyDescent="0.4">
-      <c r="A69" t="s">
-        <v>72</v>
-      </c>
-      <c r="B69" t="s">
-        <v>109</v>
-      </c>
-      <c r="C69" t="s">
-        <v>33</v>
       </c>
     </row>
   </sheetData>
@@ -2632,7 +2659,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EFD478E0-1E8A-3348-A795-503C066CAB7C}">
-  <dimension ref="A1:E152"/>
+  <dimension ref="A1:E153"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.83203125" defaultRowHeight="16" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="1" width="29.5" style="15" bestFit="1" customWidth="1"/>
@@ -2645,78 +2672,78 @@
   <sheetData>
     <row r="1" spans="1:5" ht="16.5" x14ac:dyDescent="0.4">
       <c r="A1" s="13" t="s">
+        <v>337</v>
+      </c>
+      <c r="B1" s="13" t="s">
         <v>338</v>
       </c>
-      <c r="B1" s="13" t="s">
+      <c r="C1" s="13" t="s">
         <v>339</v>
       </c>
-      <c r="C1" s="13" t="s">
+      <c r="D1" s="13" t="s">
         <v>340</v>
       </c>
-      <c r="D1" s="13" t="s">
+      <c r="E1" s="14" t="s">
         <v>341</v>
-      </c>
-      <c r="E1" s="14" t="s">
-        <v>342</v>
       </c>
     </row>
     <row r="2" spans="1:5" ht="16.5" x14ac:dyDescent="0.4">
       <c r="A2" s="16" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B2" s="17" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="C2" s="18" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="D2" s="16"/>
     </row>
     <row r="3" spans="1:5" ht="16.5" x14ac:dyDescent="0.4">
       <c r="A3" s="16" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B3" s="18" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="C3" s="18" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="D3" s="16"/>
     </row>
     <row r="4" spans="1:5" ht="16.5" x14ac:dyDescent="0.4">
       <c r="A4" s="16" t="s">
+        <v>7</v>
+      </c>
+      <c r="B4" s="18" t="s">
+        <v>114</v>
+      </c>
+      <c r="C4" s="18" t="s">
         <v>8</v>
-      </c>
-      <c r="B4" s="18" t="s">
-        <v>115</v>
-      </c>
-      <c r="C4" s="18" t="s">
-        <v>9</v>
       </c>
       <c r="D4" s="16"/>
     </row>
     <row r="5" spans="1:5" ht="16.5" x14ac:dyDescent="0.4">
       <c r="A5" s="16" t="s">
+        <v>7</v>
+      </c>
+      <c r="B5" s="18" t="s">
+        <v>115</v>
+      </c>
+      <c r="C5" s="18" t="s">
         <v>8</v>
-      </c>
-      <c r="B5" s="18" t="s">
-        <v>116</v>
-      </c>
-      <c r="C5" s="18" t="s">
-        <v>9</v>
       </c>
       <c r="D5" s="16"/>
     </row>
     <row r="6" spans="1:5" ht="16.5" x14ac:dyDescent="0.4">
       <c r="A6" s="19" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B6" s="20" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="C6" s="20" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="D6" s="19"/>
       <c r="E6" s="21"/>
@@ -2726,2051 +2753,2066 @@
         <v>1</v>
       </c>
       <c r="B7" s="23" t="s">
+        <v>381</v>
+      </c>
+      <c r="C7" s="23" t="s">
+        <v>384</v>
+      </c>
+      <c r="D7" s="22" t="s">
+        <v>381</v>
+      </c>
+      <c r="E7" s="22"/>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A8" s="34" t="s">
+        <v>1</v>
+      </c>
+      <c r="B8" s="35" t="s">
+        <v>382</v>
+      </c>
+      <c r="C8" s="35" t="s">
+        <v>383</v>
+      </c>
+      <c r="D8" s="34" t="s">
+        <v>382</v>
+      </c>
+      <c r="E8" s="34"/>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A9" s="15" t="s">
+        <v>1</v>
+      </c>
+      <c r="B9" s="18" t="s">
         <v>2</v>
       </c>
-      <c r="C7" s="23" t="s">
+      <c r="C9" s="18" t="s">
+        <v>6</v>
+      </c>
+      <c r="D9" s="15" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A10" s="21" t="s">
+        <v>1</v>
+      </c>
+      <c r="B10" s="20" t="s">
+        <v>3</v>
+      </c>
+      <c r="C10" s="20" t="s">
         <v>5</v>
       </c>
-      <c r="D7" s="22" t="s">
-        <v>2</v>
-      </c>
-      <c r="E7" s="22"/>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.4">
-      <c r="A8" s="15" t="s">
-        <v>1</v>
-      </c>
-      <c r="B8" s="18" t="s">
+      <c r="D10" s="21" t="s">
         <v>3</v>
       </c>
-      <c r="C8" s="18" t="s">
-        <v>7</v>
-      </c>
-      <c r="D8" s="15" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.4">
-      <c r="A9" s="21" t="s">
-        <v>1</v>
-      </c>
-      <c r="B9" s="20" t="s">
-        <v>4</v>
-      </c>
-      <c r="C9" s="20" t="s">
-        <v>6</v>
-      </c>
-      <c r="D9" s="21" t="s">
-        <v>4</v>
-      </c>
-      <c r="E9" s="21"/>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.4">
-      <c r="A10" s="22" t="s">
+      <c r="E10" s="21"/>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A11" s="22" t="s">
+        <v>9</v>
+      </c>
+      <c r="B11" s="23" t="s">
         <v>10</v>
       </c>
-      <c r="B10" s="23" t="s">
+      <c r="C11" s="24" t="s">
+        <v>53</v>
+      </c>
+      <c r="D11" s="25" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A12" s="21" t="s">
+        <v>9</v>
+      </c>
+      <c r="B12" s="20" t="s">
         <v>11</v>
       </c>
-      <c r="C10" s="24" t="s">
+      <c r="C12" s="26" t="s">
+        <v>52</v>
+      </c>
+      <c r="D12" s="27" t="s">
+        <v>128</v>
+      </c>
+      <c r="E12" s="21"/>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A13" s="22" t="s">
         <v>54</v>
       </c>
-      <c r="D10" s="25" t="s">
-        <v>128</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.4">
-      <c r="A11" s="21" t="s">
-        <v>10</v>
-      </c>
-      <c r="B11" s="20" t="s">
-        <v>12</v>
-      </c>
-      <c r="C11" s="26" t="s">
-        <v>53</v>
-      </c>
-      <c r="D11" s="27" t="s">
-        <v>129</v>
-      </c>
-      <c r="E11" s="21"/>
-    </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.4">
-      <c r="A12" s="22" t="s">
-        <v>55</v>
-      </c>
-      <c r="B12" s="23" t="s">
-        <v>45</v>
-      </c>
-      <c r="C12" s="23" t="s">
-        <v>27</v>
-      </c>
-      <c r="D12" s="22" t="s">
+      <c r="B13" s="23" t="s">
+        <v>44</v>
+      </c>
+      <c r="C13" s="23" t="s">
+        <v>26</v>
+      </c>
+      <c r="D13" s="22" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A14" s="21" t="s">
+        <v>54</v>
+      </c>
+      <c r="B14" s="20" t="s">
+        <v>46</v>
+      </c>
+      <c r="C14" s="20" t="s">
+        <v>29</v>
+      </c>
+      <c r="D14" s="21" t="s">
         <v>131</v>
       </c>
-    </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.4">
-      <c r="A13" s="21" t="s">
-        <v>55</v>
-      </c>
-      <c r="B13" s="20" t="s">
-        <v>47</v>
-      </c>
-      <c r="C13" s="20" t="s">
-        <v>30</v>
-      </c>
-      <c r="D13" s="21" t="s">
-        <v>132</v>
-      </c>
-      <c r="E13" s="21"/>
-    </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.4">
-      <c r="A14" s="22" t="s">
-        <v>73</v>
-      </c>
-      <c r="B14" s="23" t="s">
-        <v>57</v>
-      </c>
-      <c r="C14" s="23" t="s">
-        <v>27</v>
-      </c>
-      <c r="D14" s="22"/>
-      <c r="E14" s="22"/>
+      <c r="E14" s="21"/>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.4">
-      <c r="A15" s="15" t="s">
-        <v>73</v>
-      </c>
-      <c r="B15" s="18" t="s">
-        <v>58</v>
-      </c>
-      <c r="C15" s="18" t="s">
+      <c r="A15" s="22" t="s">
+        <v>72</v>
+      </c>
+      <c r="B15" s="23" t="s">
         <v>56</v>
       </c>
+      <c r="C15" s="23" t="s">
+        <v>26</v>
+      </c>
+      <c r="D15" s="22"/>
+      <c r="E15" s="22"/>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A16" s="15" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B16" s="18" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="C16" s="18" t="s">
-        <v>29</v>
+        <v>55</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A17" s="15" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B17" s="18" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="C17" s="18" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A18" s="15" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B18" s="18" t="s">
-        <v>156</v>
+        <v>59</v>
       </c>
       <c r="C18" s="18" t="s">
-        <v>159</v>
+        <v>25</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.4">
-      <c r="A19" s="21" t="s">
-        <v>73</v>
-      </c>
-      <c r="B19" s="20" t="s">
-        <v>61</v>
-      </c>
-      <c r="C19" s="20" t="s">
-        <v>30</v>
-      </c>
-      <c r="D19" s="21"/>
-      <c r="E19" s="21"/>
+      <c r="A19" s="15" t="s">
+        <v>72</v>
+      </c>
+      <c r="B19" s="18" t="s">
+        <v>155</v>
+      </c>
+      <c r="C19" s="18" t="s">
+        <v>158</v>
+      </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.4">
-      <c r="A20" s="22" t="s">
+      <c r="A20" s="21" t="s">
+        <v>72</v>
+      </c>
+      <c r="B20" s="20" t="s">
+        <v>60</v>
+      </c>
+      <c r="C20" s="20" t="s">
+        <v>29</v>
+      </c>
+      <c r="D20" s="21"/>
+      <c r="E20" s="21"/>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A21" s="22" t="s">
+        <v>12</v>
+      </c>
+      <c r="B21" s="23" t="s">
         <v>13</v>
       </c>
-      <c r="B20" s="23" t="s">
-        <v>14</v>
-      </c>
-      <c r="C20" s="23" t="s">
-        <v>37</v>
-      </c>
-      <c r="D20" s="22"/>
-      <c r="E20" s="22"/>
-    </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.4">
-      <c r="A21" s="15" t="s">
-        <v>13</v>
-      </c>
-      <c r="B21" s="18" t="s">
-        <v>15</v>
-      </c>
-      <c r="C21" s="18" t="s">
-        <v>38</v>
-      </c>
-      <c r="E21" s="15" t="s">
-        <v>168</v>
-      </c>
+      <c r="C21" s="23" t="s">
+        <v>36</v>
+      </c>
+      <c r="D21" s="22"/>
+      <c r="E21" s="22"/>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A22" s="15" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B22" s="18" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="C22" s="18" t="s">
-        <v>39</v>
-      </c>
-      <c r="D22" s="15" t="s">
-        <v>136</v>
+        <v>37</v>
+      </c>
+      <c r="E22" s="15" t="s">
+        <v>167</v>
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A23" s="15" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B23" s="18" t="s">
-        <v>169</v>
+        <v>15</v>
       </c>
       <c r="C23" s="18" t="s">
-        <v>170</v>
+        <v>38</v>
+      </c>
+      <c r="D23" s="15" t="s">
+        <v>135</v>
       </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A24" s="15" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B24" s="18" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
       <c r="C24" s="18" t="s">
-        <v>172</v>
+        <v>169</v>
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A25" s="15" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B25" s="18" t="s">
-        <v>18</v>
+        <v>170</v>
       </c>
       <c r="C25" s="18" t="s">
-        <v>40</v>
-      </c>
-      <c r="D25" s="15" t="s">
-        <v>133</v>
+        <v>171</v>
       </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A26" s="15" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B26" s="18" t="s">
-        <v>351</v>
+        <v>17</v>
       </c>
       <c r="C26" s="18" t="s">
-        <v>352</v>
+        <v>39</v>
       </c>
       <c r="D26" s="15" t="s">
-        <v>354</v>
+        <v>132</v>
       </c>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A27" s="15" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B27" s="18" t="s">
         <v>350</v>
       </c>
       <c r="C27" s="18" t="s">
+        <v>351</v>
+      </c>
+      <c r="D27" s="15" t="s">
         <v>353</v>
-      </c>
-      <c r="D27" s="15" t="s">
-        <v>355</v>
       </c>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A28" s="15" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B28" s="18" t="s">
-        <v>359</v>
+        <v>349</v>
       </c>
       <c r="C28" s="18" t="s">
-        <v>360</v>
+        <v>352</v>
       </c>
       <c r="D28" s="15" t="s">
-        <v>365</v>
+        <v>354</v>
       </c>
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A29" s="15" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B29" s="18" t="s">
-        <v>361</v>
+        <v>358</v>
       </c>
       <c r="C29" s="18" t="s">
-        <v>362</v>
+        <v>359</v>
       </c>
       <c r="D29" s="15" t="s">
-        <v>366</v>
+        <v>364</v>
       </c>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A30" s="15" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B30" s="18" t="s">
-        <v>363</v>
+        <v>360</v>
       </c>
       <c r="C30" s="18" t="s">
-        <v>364</v>
+        <v>361</v>
+      </c>
+      <c r="D30" s="15" t="s">
+        <v>365</v>
       </c>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A31" s="15" t="s">
-        <v>13</v>
-      </c>
-      <c r="B31" s="28" t="s">
-        <v>19</v>
-      </c>
-      <c r="C31" s="28" t="s">
-        <v>41</v>
-      </c>
-      <c r="D31" s="15" t="s">
-        <v>345</v>
+        <v>12</v>
+      </c>
+      <c r="B31" s="18" t="s">
+        <v>362</v>
+      </c>
+      <c r="C31" s="18" t="s">
+        <v>363</v>
       </c>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A32" s="15" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B32" s="28" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="C32" s="28" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="D32" s="15" t="s">
-        <v>346</v>
+        <v>344</v>
       </c>
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A33" s="15" t="s">
-        <v>13</v>
-      </c>
-      <c r="B33" s="18" t="s">
-        <v>149</v>
-      </c>
-      <c r="C33" s="18" t="s">
-        <v>173</v>
+        <v>12</v>
+      </c>
+      <c r="B33" s="28" t="s">
+        <v>19</v>
+      </c>
+      <c r="C33" s="28" t="s">
+        <v>41</v>
       </c>
       <c r="D33" s="15" t="s">
-        <v>367</v>
-      </c>
-      <c r="E33" s="15" t="s">
-        <v>150</v>
+        <v>345</v>
       </c>
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A34" s="15" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B34" s="18" t="s">
-        <v>23</v>
+        <v>148</v>
       </c>
       <c r="C34" s="18" t="s">
-        <v>34</v>
+        <v>172</v>
+      </c>
+      <c r="D34" s="15" t="s">
+        <v>366</v>
+      </c>
+      <c r="E34" s="15" t="s">
+        <v>149</v>
       </c>
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A35" s="15" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B35" s="18" t="s">
+        <v>22</v>
+      </c>
+      <c r="C35" s="18" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="36" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A36" s="15" t="s">
+        <v>12</v>
+      </c>
+      <c r="B36" s="18" t="s">
+        <v>23</v>
+      </c>
+      <c r="C36" s="18" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="37" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A37" s="21" t="s">
+        <v>12</v>
+      </c>
+      <c r="B37" s="20" t="s">
         <v>24</v>
       </c>
-      <c r="C35" s="18" t="s">
+      <c r="C37" s="20" t="s">
         <v>35</v>
       </c>
-    </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.4">
-      <c r="A36" s="21" t="s">
-        <v>13</v>
-      </c>
-      <c r="B36" s="20" t="s">
-        <v>25</v>
-      </c>
-      <c r="C36" s="20" t="s">
-        <v>36</v>
-      </c>
-      <c r="D36" s="21" t="s">
+      <c r="D37" s="21" t="s">
+        <v>136</v>
+      </c>
+      <c r="E37" s="21"/>
+    </row>
+    <row r="38" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A38" s="22" t="s">
+        <v>346</v>
+      </c>
+      <c r="B38" s="23" t="s">
+        <v>48</v>
+      </c>
+      <c r="C38" s="23" t="s">
+        <v>50</v>
+      </c>
+      <c r="D38" s="22" t="s">
         <v>137</v>
       </c>
-      <c r="E36" s="21"/>
-    </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.4">
-      <c r="A37" s="22" t="s">
-        <v>347</v>
-      </c>
-      <c r="B37" s="23" t="s">
+      <c r="E38" s="22"/>
+    </row>
+    <row r="39" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A39" s="15" t="s">
+        <v>346</v>
+      </c>
+      <c r="B39" s="18" t="s">
         <v>49</v>
       </c>
-      <c r="C37" s="23" t="s">
+      <c r="C39" s="18" t="s">
         <v>51</v>
       </c>
-      <c r="D37" s="22" t="s">
+      <c r="D39" s="15" t="s">
         <v>138</v>
       </c>
-      <c r="E37" s="22"/>
-    </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.4">
-      <c r="A38" s="15" t="s">
-        <v>347</v>
-      </c>
-      <c r="B38" s="18" t="s">
-        <v>50</v>
-      </c>
-      <c r="C38" s="18" t="s">
-        <v>52</v>
-      </c>
-      <c r="D38" s="15" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.4">
-      <c r="A39" s="21" t="s">
-        <v>347</v>
-      </c>
-      <c r="B39" s="20" t="s">
-        <v>25</v>
-      </c>
-      <c r="C39" s="20" t="s">
-        <v>36</v>
-      </c>
-      <c r="D39" s="21" t="s">
-        <v>137</v>
-      </c>
-      <c r="E39" s="21"/>
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.4">
-      <c r="A40" s="22" t="s">
-        <v>74</v>
-      </c>
-      <c r="B40" s="23" t="s">
-        <v>46</v>
-      </c>
-      <c r="C40" s="23" t="s">
-        <v>27</v>
-      </c>
-      <c r="D40" s="22" t="s">
-        <v>131</v>
-      </c>
-      <c r="E40" s="22"/>
+      <c r="A40" s="21" t="s">
+        <v>346</v>
+      </c>
+      <c r="B40" s="20" t="s">
+        <v>24</v>
+      </c>
+      <c r="C40" s="20" t="s">
+        <v>35</v>
+      </c>
+      <c r="D40" s="21" t="s">
+        <v>136</v>
+      </c>
+      <c r="E40" s="21"/>
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.4">
-      <c r="A41" s="15" t="s">
-        <v>74</v>
-      </c>
-      <c r="B41" s="18" t="s">
-        <v>62</v>
-      </c>
-      <c r="C41" s="18" t="s">
+      <c r="A41" s="22" t="s">
+        <v>73</v>
+      </c>
+      <c r="B41" s="23" t="s">
+        <v>45</v>
+      </c>
+      <c r="C41" s="23" t="s">
         <v>26</v>
       </c>
-      <c r="D41" s="15" t="s">
-        <v>140</v>
-      </c>
+      <c r="D41" s="22" t="s">
+        <v>130</v>
+      </c>
+      <c r="E41" s="22"/>
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A42" s="15" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B42" s="18" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="C42" s="18" t="s">
-        <v>65</v>
+        <v>25</v>
       </c>
       <c r="D42" s="15" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
     </row>
     <row r="43" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A43" s="15" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B43" s="18" t="s">
+        <v>62</v>
+      </c>
+      <c r="C43" s="18" t="s">
         <v>64</v>
       </c>
-      <c r="C43" s="18" t="s">
-        <v>30</v>
-      </c>
       <c r="D43" s="15" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
     </row>
     <row r="44" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A44" s="15" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B44" s="18" t="s">
-        <v>174</v>
+        <v>63</v>
       </c>
       <c r="C44" s="18" t="s">
-        <v>175</v>
+        <v>29</v>
       </c>
       <c r="D44" s="15" t="s">
-        <v>176</v>
+        <v>141</v>
       </c>
     </row>
     <row r="45" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A45" s="15" t="s">
+        <v>73</v>
+      </c>
+      <c r="B45" s="18" t="s">
+        <v>173</v>
+      </c>
+      <c r="C45" s="18" t="s">
+        <v>174</v>
+      </c>
+      <c r="D45" s="15" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="46" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A46" s="15" t="s">
+        <v>73</v>
+      </c>
+      <c r="B46" s="18" t="s">
+        <v>24</v>
+      </c>
+      <c r="C46" s="18" t="s">
+        <v>35</v>
+      </c>
+      <c r="D46" s="21" t="s">
+        <v>136</v>
+      </c>
+      <c r="E46" s="21"/>
+    </row>
+    <row r="47" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A47" s="22" t="s">
+        <v>65</v>
+      </c>
+      <c r="B47" s="23" t="s">
+        <v>66</v>
+      </c>
+      <c r="C47" s="23" t="s">
+        <v>67</v>
+      </c>
+      <c r="D47" s="22" t="s">
+        <v>342</v>
+      </c>
+      <c r="E47" s="22"/>
+    </row>
+    <row r="48" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A48" s="15" t="s">
+        <v>65</v>
+      </c>
+      <c r="B48" s="18" t="s">
+        <v>68</v>
+      </c>
+      <c r="C48" s="18" t="s">
+        <v>69</v>
+      </c>
+      <c r="D48" s="15" t="s">
+        <v>343</v>
+      </c>
+    </row>
+    <row r="49" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A49" s="21" t="s">
+        <v>65</v>
+      </c>
+      <c r="B49" s="20" t="s">
+        <v>24</v>
+      </c>
+      <c r="C49" s="20" t="s">
+        <v>35</v>
+      </c>
+      <c r="D49" s="21" t="s">
+        <v>130</v>
+      </c>
+      <c r="E49" s="21"/>
+    </row>
+    <row r="50" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A50" s="22" t="s">
         <v>74</v>
       </c>
-      <c r="B45" s="18" t="s">
-        <v>25</v>
-      </c>
-      <c r="C45" s="18" t="s">
-        <v>36</v>
-      </c>
-      <c r="D45" s="21" t="s">
-        <v>137</v>
-      </c>
-      <c r="E45" s="21"/>
-    </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.4">
-      <c r="A46" s="22" t="s">
-        <v>66</v>
-      </c>
-      <c r="B46" s="23" t="s">
-        <v>67</v>
-      </c>
-      <c r="C46" s="23" t="s">
-        <v>68</v>
-      </c>
-      <c r="D46" s="22" t="s">
-        <v>343</v>
-      </c>
-      <c r="E46" s="22"/>
-    </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.4">
-      <c r="A47" s="15" t="s">
-        <v>66</v>
-      </c>
-      <c r="B47" s="18" t="s">
-        <v>69</v>
-      </c>
-      <c r="C47" s="18" t="s">
+      <c r="B50" s="23" t="s">
+        <v>75</v>
+      </c>
+      <c r="C50" s="23" t="s">
+        <v>77</v>
+      </c>
+      <c r="D50" s="22" t="s">
+        <v>144</v>
+      </c>
+      <c r="E50" s="22"/>
+    </row>
+    <row r="51" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A51" s="15" t="s">
+        <v>74</v>
+      </c>
+      <c r="B51" s="18" t="s">
+        <v>76</v>
+      </c>
+      <c r="C51" s="18" t="s">
+        <v>78</v>
+      </c>
+      <c r="D51" s="15" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="52" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A52" s="21" t="s">
+        <v>74</v>
+      </c>
+      <c r="B52" s="20" t="s">
+        <v>24</v>
+      </c>
+      <c r="C52" s="20" t="s">
+        <v>35</v>
+      </c>
+      <c r="D52" s="21" t="s">
+        <v>136</v>
+      </c>
+      <c r="E52" s="21"/>
+    </row>
+    <row r="53" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A53" s="22" t="s">
         <v>70</v>
       </c>
-      <c r="D47" s="15" t="s">
-        <v>344</v>
-      </c>
-    </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.4">
-      <c r="A48" s="21" t="s">
-        <v>66</v>
-      </c>
-      <c r="B48" s="20" t="s">
-        <v>25</v>
-      </c>
-      <c r="C48" s="20" t="s">
-        <v>36</v>
-      </c>
-      <c r="D48" s="21" t="s">
-        <v>131</v>
-      </c>
-      <c r="E48" s="21"/>
-    </row>
-    <row r="49" spans="1:5" x14ac:dyDescent="0.4">
-      <c r="A49" s="22" t="s">
-        <v>75</v>
-      </c>
-      <c r="B49" s="23" t="s">
-        <v>76</v>
-      </c>
-      <c r="C49" s="23" t="s">
-        <v>78</v>
-      </c>
-      <c r="D49" s="22" t="s">
-        <v>145</v>
-      </c>
-      <c r="E49" s="22"/>
-    </row>
-    <row r="50" spans="1:5" x14ac:dyDescent="0.4">
-      <c r="A50" s="15" t="s">
-        <v>75</v>
-      </c>
-      <c r="B50" s="18" t="s">
-        <v>77</v>
-      </c>
-      <c r="C50" s="18" t="s">
+      <c r="B53" s="23" t="s">
         <v>79</v>
       </c>
-      <c r="D50" s="15" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="51" spans="1:5" x14ac:dyDescent="0.4">
-      <c r="A51" s="21" t="s">
-        <v>75</v>
-      </c>
-      <c r="B51" s="20" t="s">
-        <v>25</v>
-      </c>
-      <c r="C51" s="20" t="s">
-        <v>36</v>
-      </c>
-      <c r="D51" s="21" t="s">
-        <v>137</v>
-      </c>
-      <c r="E51" s="21"/>
-    </row>
-    <row r="52" spans="1:5" x14ac:dyDescent="0.4">
-      <c r="A52" s="22" t="s">
-        <v>71</v>
-      </c>
-      <c r="B52" s="23" t="s">
+      <c r="C53" s="23" t="s">
+        <v>79</v>
+      </c>
+      <c r="D53" s="15" t="s">
+        <v>176</v>
+      </c>
+      <c r="E53" s="22"/>
+    </row>
+    <row r="54" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A54" s="15" t="s">
+        <v>70</v>
+      </c>
+      <c r="B54" s="18" t="s">
         <v>80</v>
       </c>
-      <c r="C52" s="23" t="s">
-        <v>80</v>
-      </c>
-      <c r="D52" s="15" t="s">
+      <c r="C54" s="18" t="s">
+        <v>95</v>
+      </c>
+      <c r="D54" s="15" t="s">
         <v>177</v>
       </c>
-      <c r="E52" s="22"/>
-    </row>
-    <row r="53" spans="1:5" x14ac:dyDescent="0.4">
-      <c r="A53" s="15" t="s">
-        <v>71</v>
-      </c>
-      <c r="B53" s="18" t="s">
-        <v>81</v>
-      </c>
-      <c r="C53" s="18" t="s">
-        <v>96</v>
-      </c>
-      <c r="D53" s="15" t="s">
+    </row>
+    <row r="55" spans="1:5" ht="16.5" x14ac:dyDescent="0.4">
+      <c r="A55" s="29" t="s">
+        <v>70</v>
+      </c>
+      <c r="B55" s="30" t="s">
+        <v>150</v>
+      </c>
+      <c r="C55" s="30" t="s">
+        <v>151</v>
+      </c>
+      <c r="D55" s="15" t="s">
         <v>178</v>
       </c>
-    </row>
-    <row r="54" spans="1:5" ht="16.5" x14ac:dyDescent="0.4">
-      <c r="A54" s="29" t="s">
-        <v>71</v>
-      </c>
-      <c r="B54" s="30" t="s">
-        <v>151</v>
-      </c>
-      <c r="C54" s="30" t="s">
+      <c r="E55" s="29" t="s">
         <v>152</v>
-      </c>
-      <c r="D54" s="15" t="s">
-        <v>179</v>
-      </c>
-      <c r="E54" s="29" t="s">
-        <v>153</v>
-      </c>
-    </row>
-    <row r="55" spans="1:5" ht="16.5" x14ac:dyDescent="0.4">
-      <c r="A55" s="15" t="s">
-        <v>71</v>
-      </c>
-      <c r="B55" s="18" t="s">
-        <v>83</v>
-      </c>
-      <c r="C55" s="18" t="s">
-        <v>121</v>
-      </c>
-      <c r="D55" s="15" t="s">
-        <v>160</v>
-      </c>
-      <c r="E55" s="29" t="s">
-        <v>154</v>
       </c>
     </row>
     <row r="56" spans="1:5" ht="16.5" x14ac:dyDescent="0.4">
       <c r="A56" s="15" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B56" s="18" t="s">
+        <v>82</v>
+      </c>
+      <c r="C56" s="18" t="s">
+        <v>120</v>
+      </c>
+      <c r="D56" s="15" t="s">
+        <v>159</v>
+      </c>
+      <c r="E56" s="29" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="57" spans="1:5" ht="16.5" x14ac:dyDescent="0.4">
+      <c r="A57" s="15" t="s">
+        <v>70</v>
+      </c>
+      <c r="B57" s="18" t="s">
+        <v>373</v>
+      </c>
+      <c r="C57" s="18" t="s">
         <v>374</v>
       </c>
-      <c r="C56" s="18" t="s">
+      <c r="D57" s="15" t="s">
         <v>375</v>
       </c>
-      <c r="D56" s="15" t="s">
-        <v>376</v>
-      </c>
-      <c r="E56" s="29"/>
-    </row>
-    <row r="57" spans="1:5" x14ac:dyDescent="0.4">
-      <c r="A57" s="15" t="s">
-        <v>71</v>
-      </c>
-      <c r="B57" s="18" t="s">
-        <v>93</v>
-      </c>
-      <c r="C57" s="18" t="s">
-        <v>122</v>
-      </c>
-      <c r="D57" s="15" t="s">
-        <v>165</v>
-      </c>
+      <c r="E57" s="29"/>
     </row>
     <row r="58" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A58" s="15" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B58" s="18" t="s">
-        <v>84</v>
+        <v>92</v>
       </c>
       <c r="C58" s="18" t="s">
-        <v>98</v>
+        <v>121</v>
       </c>
       <c r="D58" s="15" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
     </row>
     <row r="59" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A59" s="15" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B59" s="18" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="C59" s="18" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="D59" s="15" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
     </row>
     <row r="60" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A60" s="15" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B60" s="18" t="s">
-        <v>91</v>
+        <v>84</v>
       </c>
       <c r="C60" s="18" t="s">
-        <v>104</v>
+        <v>98</v>
       </c>
       <c r="D60" s="15" t="s">
-        <v>166</v>
+        <v>161</v>
       </c>
     </row>
     <row r="61" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A61" s="15" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B61" s="18" t="s">
         <v>90</v>
       </c>
       <c r="C61" s="18" t="s">
-        <v>90</v>
+        <v>103</v>
       </c>
       <c r="D61" s="15" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
     </row>
     <row r="62" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A62" s="15" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B62" s="18" t="s">
-        <v>82</v>
+        <v>89</v>
       </c>
       <c r="C62" s="18" t="s">
-        <v>97</v>
+        <v>89</v>
       </c>
       <c r="D62" s="15" t="s">
-        <v>180</v>
+        <v>166</v>
       </c>
     </row>
     <row r="63" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A63" s="15" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B63" s="18" t="s">
-        <v>92</v>
+        <v>81</v>
       </c>
       <c r="C63" s="18" t="s">
-        <v>105</v>
+        <v>96</v>
       </c>
       <c r="D63" s="15" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
     </row>
     <row r="64" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A64" s="15" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B64" s="18" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="C64" s="18" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="D64" s="15" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
     </row>
     <row r="65" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A65" s="15" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B65" s="18" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="C65" s="18" t="s">
-        <v>95</v>
+        <v>105</v>
       </c>
       <c r="D65" s="15" t="s">
-        <v>183</v>
-      </c>
-    </row>
-    <row r="66" spans="1:5" ht="16.5" x14ac:dyDescent="0.4">
-      <c r="A66" s="29" t="s">
-        <v>71</v>
-      </c>
-      <c r="B66" s="30" t="s">
-        <v>5</v>
-      </c>
-      <c r="C66" s="30" t="s">
-        <v>107</v>
+        <v>181</v>
+      </c>
+    </row>
+    <row r="66" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A66" s="15" t="s">
+        <v>70</v>
+      </c>
+      <c r="B66" s="18" t="s">
+        <v>94</v>
+      </c>
+      <c r="C66" s="18" t="s">
+        <v>94</v>
       </c>
       <c r="D66" s="15" t="s">
-        <v>184</v>
-      </c>
-      <c r="E66" s="29" t="s">
-        <v>157</v>
+        <v>182</v>
       </c>
     </row>
     <row r="67" spans="1:5" ht="16.5" x14ac:dyDescent="0.4">
       <c r="A67" s="29" t="s">
+        <v>70</v>
+      </c>
+      <c r="B67" s="30" t="s">
+        <v>4</v>
+      </c>
+      <c r="C67" s="30" t="s">
+        <v>106</v>
+      </c>
+      <c r="D67" s="15" t="s">
+        <v>183</v>
+      </c>
+      <c r="E67" s="29" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="68" spans="1:5" ht="16.5" x14ac:dyDescent="0.4">
+      <c r="A68" s="29" t="s">
+        <v>70</v>
+      </c>
+      <c r="B68" s="30" t="s">
+        <v>355</v>
+      </c>
+      <c r="C68" s="30" t="s">
+        <v>356</v>
+      </c>
+      <c r="D68" s="15" t="s">
+        <v>357</v>
+      </c>
+      <c r="E68" s="29"/>
+    </row>
+    <row r="69" spans="1:5" ht="16.5" x14ac:dyDescent="0.4">
+      <c r="A69" s="31" t="s">
+        <v>70</v>
+      </c>
+      <c r="B69" s="32" t="s">
+        <v>125</v>
+      </c>
+      <c r="C69" s="32" t="s">
+        <v>124</v>
+      </c>
+      <c r="D69" s="21" t="s">
+        <v>163</v>
+      </c>
+      <c r="E69" s="31" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="70" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A70" s="22" t="s">
         <v>71</v>
       </c>
-      <c r="B67" s="30" t="s">
-        <v>356</v>
-      </c>
-      <c r="C67" s="30" t="s">
-        <v>357</v>
-      </c>
-      <c r="D67" s="15" t="s">
-        <v>358</v>
-      </c>
-      <c r="E67" s="29"/>
-    </row>
-    <row r="68" spans="1:5" ht="16.5" x14ac:dyDescent="0.4">
-      <c r="A68" s="31" t="s">
-        <v>71</v>
-      </c>
-      <c r="B68" s="32" t="s">
-        <v>126</v>
-      </c>
-      <c r="C68" s="32" t="s">
-        <v>125</v>
-      </c>
-      <c r="D68" s="21" t="s">
-        <v>164</v>
-      </c>
-      <c r="E68" s="31" t="s">
-        <v>155</v>
-      </c>
-    </row>
-    <row r="69" spans="1:5" x14ac:dyDescent="0.4">
-      <c r="A69" s="22" t="s">
-        <v>72</v>
-      </c>
-      <c r="B69" s="23" t="s">
-        <v>108</v>
-      </c>
-      <c r="C69" s="23" t="s">
-        <v>110</v>
-      </c>
-      <c r="D69" s="15" t="s">
-        <v>185</v>
-      </c>
-      <c r="E69" s="22"/>
-    </row>
-    <row r="70" spans="1:5" x14ac:dyDescent="0.4">
-      <c r="A70" s="15" t="s">
-        <v>72</v>
-      </c>
-      <c r="B70" s="18" t="s">
-        <v>82</v>
-      </c>
-      <c r="C70" s="18" t="s">
-        <v>97</v>
+      <c r="B70" s="23" t="s">
+        <v>107</v>
+      </c>
+      <c r="C70" s="23" t="s">
+        <v>109</v>
       </c>
       <c r="D70" s="15" t="s">
-        <v>180</v>
-      </c>
+        <v>184</v>
+      </c>
+      <c r="E70" s="22"/>
     </row>
     <row r="71" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A71" s="15" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B71" s="18" t="s">
-        <v>22</v>
+        <v>81</v>
       </c>
       <c r="C71" s="18" t="s">
-        <v>32</v>
+        <v>96</v>
       </c>
       <c r="D71" s="15" t="s">
-        <v>186</v>
+        <v>179</v>
       </c>
     </row>
     <row r="72" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A72" s="15" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B72" s="18" t="s">
-        <v>368</v>
+        <v>21</v>
       </c>
       <c r="C72" s="18" t="s">
-        <v>370</v>
+        <v>31</v>
       </c>
       <c r="D72" s="15" t="s">
-        <v>372</v>
+        <v>185</v>
       </c>
     </row>
     <row r="73" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A73" s="15" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B73" s="18" t="s">
+        <v>367</v>
+      </c>
+      <c r="C73" s="18" t="s">
         <v>369</v>
       </c>
-      <c r="C73" s="18" t="s">
+      <c r="D73" s="15" t="s">
         <v>371</v>
       </c>
-      <c r="D73" s="15" t="s">
-        <v>373</v>
-      </c>
-    </row>
-    <row r="74" spans="1:5" ht="16.5" x14ac:dyDescent="0.4">
+    </row>
+    <row r="74" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A74" s="15" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B74" s="18" t="s">
-        <v>120</v>
+        <v>368</v>
       </c>
       <c r="C74" s="18" t="s">
-        <v>31</v>
+        <v>370</v>
       </c>
       <c r="D74" s="15" t="s">
-        <v>163</v>
-      </c>
-      <c r="E74" s="29" t="s">
+        <v>372</v>
+      </c>
+    </row>
+    <row r="75" spans="1:5" ht="16.5" x14ac:dyDescent="0.4">
+      <c r="A75" s="15" t="s">
+        <v>71</v>
+      </c>
+      <c r="B75" s="18" t="s">
+        <v>119</v>
+      </c>
+      <c r="C75" s="18" t="s">
+        <v>30</v>
+      </c>
+      <c r="D75" s="15" t="s">
+        <v>162</v>
+      </c>
+      <c r="E75" s="29" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="76" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A76" s="15" t="s">
+        <v>71</v>
+      </c>
+      <c r="B76" s="18" t="s">
+        <v>108</v>
+      </c>
+      <c r="C76" s="18" t="s">
+        <v>32</v>
+      </c>
+      <c r="D76" s="15" t="s">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="77" spans="1:5" ht="16.5" x14ac:dyDescent="0.4">
+      <c r="A77" s="15" t="s">
+        <v>71</v>
+      </c>
+      <c r="B77" s="30" t="s">
+        <v>126</v>
+      </c>
+      <c r="C77" s="30" t="s">
+        <v>126</v>
+      </c>
+      <c r="D77" s="15" t="s">
         <v>187</v>
       </c>
-    </row>
-    <row r="75" spans="1:5" x14ac:dyDescent="0.4">
-      <c r="A75" s="15" t="s">
-        <v>72</v>
-      </c>
-      <c r="B75" s="18" t="s">
-        <v>109</v>
-      </c>
-      <c r="C75" s="18" t="s">
-        <v>33</v>
-      </c>
-      <c r="D75" s="15" t="s">
+      <c r="E77" s="33"/>
+    </row>
+    <row r="78" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A78" s="21" t="s">
+        <v>71</v>
+      </c>
+      <c r="B78" s="20" t="s">
+        <v>188</v>
+      </c>
+      <c r="C78" s="20" t="s">
+        <v>189</v>
+      </c>
+      <c r="D78" s="21" t="s">
         <v>348</v>
       </c>
-    </row>
-    <row r="76" spans="1:5" ht="16.5" x14ac:dyDescent="0.4">
-      <c r="A76" s="15" t="s">
-        <v>72</v>
-      </c>
-      <c r="B76" s="30" t="s">
-        <v>127</v>
-      </c>
-      <c r="C76" s="30" t="s">
-        <v>127</v>
-      </c>
-      <c r="D76" s="15" t="s">
-        <v>188</v>
-      </c>
-      <c r="E76" s="33"/>
-    </row>
-    <row r="77" spans="1:5" x14ac:dyDescent="0.4">
-      <c r="A77" s="21" t="s">
-        <v>72</v>
-      </c>
-      <c r="B77" s="20" t="s">
-        <v>189</v>
-      </c>
-      <c r="C77" s="20" t="s">
-        <v>190</v>
-      </c>
-      <c r="D77" s="21" t="s">
-        <v>349</v>
-      </c>
-      <c r="E77" s="21"/>
-    </row>
-    <row r="78" spans="1:5" x14ac:dyDescent="0.4">
-      <c r="A78" s="15" t="s">
-        <v>191</v>
-      </c>
-      <c r="B78" s="18" t="s">
-        <v>192</v>
-      </c>
-      <c r="C78" s="18" t="s">
-        <v>192</v>
-      </c>
-      <c r="D78" s="15" t="s">
-        <v>193</v>
-      </c>
+      <c r="E78" s="21"/>
     </row>
     <row r="79" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A79" s="15" t="s">
+        <v>190</v>
+      </c>
+      <c r="B79" s="18" t="s">
         <v>191</v>
       </c>
-      <c r="B79" s="18" t="s">
-        <v>16</v>
-      </c>
       <c r="C79" s="18" t="s">
-        <v>16</v>
+        <v>191</v>
       </c>
       <c r="D79" s="15" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
     </row>
     <row r="80" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A80" s="15" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="B80" s="18" t="s">
-        <v>195</v>
+        <v>15</v>
       </c>
       <c r="C80" s="18" t="s">
-        <v>195</v>
+        <v>15</v>
       </c>
       <c r="D80" s="15" t="s">
-        <v>196</v>
+        <v>193</v>
       </c>
     </row>
     <row r="81" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A81" s="15" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="B81" s="18" t="s">
-        <v>197</v>
+        <v>194</v>
       </c>
       <c r="C81" s="18" t="s">
-        <v>197</v>
+        <v>194</v>
       </c>
       <c r="D81" s="15" t="s">
-        <v>198</v>
+        <v>195</v>
       </c>
     </row>
     <row r="82" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A82" s="15" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="B82" s="18" t="s">
-        <v>199</v>
+        <v>196</v>
       </c>
       <c r="C82" s="18" t="s">
-        <v>199</v>
+        <v>196</v>
       </c>
       <c r="D82" s="15" t="s">
-        <v>200</v>
+        <v>197</v>
       </c>
     </row>
     <row r="83" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A83" s="15" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="B83" s="18" t="s">
-        <v>201</v>
+        <v>198</v>
       </c>
       <c r="C83" s="18" t="s">
-        <v>201</v>
+        <v>198</v>
       </c>
       <c r="D83" s="15" t="s">
-        <v>202</v>
+        <v>199</v>
       </c>
     </row>
     <row r="84" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A84" s="15" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="B84" s="18" t="s">
-        <v>203</v>
+        <v>200</v>
       </c>
       <c r="C84" s="18" t="s">
-        <v>203</v>
+        <v>200</v>
       </c>
       <c r="D84" s="15" t="s">
-        <v>204</v>
+        <v>201</v>
       </c>
     </row>
     <row r="85" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A85" s="15" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="B85" s="18" t="s">
-        <v>205</v>
+        <v>202</v>
       </c>
       <c r="C85" s="18" t="s">
-        <v>205</v>
+        <v>202</v>
       </c>
       <c r="D85" s="15" t="s">
-        <v>206</v>
+        <v>203</v>
       </c>
     </row>
     <row r="86" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A86" s="15" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="B86" s="18" t="s">
-        <v>207</v>
+        <v>204</v>
       </c>
       <c r="C86" s="18" t="s">
-        <v>207</v>
+        <v>204</v>
       </c>
       <c r="D86" s="15" t="s">
-        <v>208</v>
+        <v>205</v>
       </c>
     </row>
     <row r="87" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A87" s="15" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="B87" s="18" t="s">
-        <v>209</v>
+        <v>206</v>
       </c>
       <c r="C87" s="18" t="s">
-        <v>209</v>
+        <v>206</v>
       </c>
       <c r="D87" s="15" t="s">
-        <v>210</v>
+        <v>207</v>
       </c>
     </row>
     <row r="88" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A88" s="15" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="B88" s="18" t="s">
-        <v>211</v>
+        <v>208</v>
       </c>
       <c r="C88" s="18" t="s">
-        <v>211</v>
+        <v>208</v>
       </c>
       <c r="D88" s="15" t="s">
-        <v>212</v>
+        <v>209</v>
       </c>
     </row>
     <row r="89" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A89" s="15" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="B89" s="18" t="s">
-        <v>213</v>
+        <v>210</v>
       </c>
       <c r="C89" s="18" t="s">
-        <v>213</v>
+        <v>210</v>
       </c>
       <c r="D89" s="15" t="s">
-        <v>214</v>
+        <v>211</v>
       </c>
     </row>
     <row r="90" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A90" s="15" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="B90" s="18" t="s">
-        <v>215</v>
+        <v>212</v>
       </c>
       <c r="C90" s="18" t="s">
-        <v>215</v>
+        <v>212</v>
       </c>
       <c r="D90" s="15" t="s">
-        <v>216</v>
+        <v>213</v>
       </c>
     </row>
     <row r="91" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A91" s="15" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="B91" s="18" t="s">
-        <v>217</v>
+        <v>214</v>
       </c>
       <c r="C91" s="18" t="s">
-        <v>217</v>
+        <v>214</v>
       </c>
       <c r="D91" s="15" t="s">
-        <v>218</v>
+        <v>215</v>
       </c>
     </row>
     <row r="92" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A92" s="15" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="B92" s="18" t="s">
-        <v>219</v>
+        <v>216</v>
       </c>
       <c r="C92" s="18" t="s">
-        <v>219</v>
+        <v>216</v>
       </c>
       <c r="D92" s="15" t="s">
-        <v>220</v>
+        <v>217</v>
       </c>
     </row>
     <row r="93" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A93" s="15" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="B93" s="18" t="s">
-        <v>221</v>
+        <v>218</v>
       </c>
       <c r="C93" s="18" t="s">
-        <v>221</v>
+        <v>218</v>
       </c>
       <c r="D93" s="15" t="s">
-        <v>222</v>
+        <v>219</v>
       </c>
     </row>
     <row r="94" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A94" s="15" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="B94" s="18" t="s">
-        <v>223</v>
+        <v>220</v>
       </c>
       <c r="C94" s="18" t="s">
-        <v>223</v>
+        <v>220</v>
       </c>
       <c r="D94" s="15" t="s">
-        <v>224</v>
+        <v>221</v>
       </c>
     </row>
     <row r="95" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A95" s="15" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="B95" s="18" t="s">
-        <v>225</v>
+        <v>222</v>
       </c>
       <c r="C95" s="18" t="s">
-        <v>225</v>
+        <v>222</v>
       </c>
       <c r="D95" s="15" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
     </row>
     <row r="96" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A96" s="15" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="B96" s="18" t="s">
-        <v>227</v>
+        <v>224</v>
       </c>
       <c r="C96" s="18" t="s">
-        <v>227</v>
+        <v>224</v>
       </c>
       <c r="D96" s="15" t="s">
-        <v>228</v>
+        <v>225</v>
       </c>
     </row>
     <row r="97" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A97" s="15" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="B97" s="18" t="s">
-        <v>229</v>
+        <v>226</v>
       </c>
       <c r="C97" s="18" t="s">
-        <v>229</v>
+        <v>226</v>
       </c>
       <c r="D97" s="15" t="s">
-        <v>230</v>
+        <v>227</v>
       </c>
     </row>
     <row r="98" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A98" s="15" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="B98" s="18" t="s">
-        <v>231</v>
+        <v>228</v>
       </c>
       <c r="C98" s="18" t="s">
-        <v>231</v>
+        <v>228</v>
       </c>
       <c r="D98" s="15" t="s">
-        <v>232</v>
+        <v>229</v>
       </c>
     </row>
     <row r="99" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A99" s="15" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="B99" s="18" t="s">
-        <v>233</v>
+        <v>230</v>
       </c>
       <c r="C99" s="18" t="s">
-        <v>233</v>
+        <v>230</v>
       </c>
       <c r="D99" s="15" t="s">
-        <v>234</v>
+        <v>231</v>
       </c>
     </row>
     <row r="100" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A100" s="15" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="B100" s="18" t="s">
-        <v>235</v>
+        <v>232</v>
       </c>
       <c r="C100" s="18" t="s">
-        <v>235</v>
+        <v>232</v>
       </c>
       <c r="D100" s="15" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
     </row>
     <row r="101" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A101" s="15" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="B101" s="18" t="s">
-        <v>237</v>
+        <v>234</v>
       </c>
       <c r="C101" s="18" t="s">
-        <v>237</v>
+        <v>234</v>
       </c>
       <c r="D101" s="15" t="s">
-        <v>238</v>
+        <v>235</v>
       </c>
     </row>
     <row r="102" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A102" s="15" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="B102" s="18" t="s">
+        <v>236</v>
+      </c>
+      <c r="C102" s="18" t="s">
+        <v>236</v>
+      </c>
+      <c r="D102" s="15" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="103" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A103" s="15" t="s">
+        <v>190</v>
+      </c>
+      <c r="B103" s="18" t="s">
+        <v>238</v>
+      </c>
+      <c r="C103" s="18" t="s">
+        <v>238</v>
+      </c>
+      <c r="D103" s="15" t="s">
         <v>239</v>
       </c>
-      <c r="C102" s="18" t="s">
-        <v>239</v>
-      </c>
-      <c r="D102" s="15" t="s">
+    </row>
+    <row r="104" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A104" s="21" t="s">
+        <v>190</v>
+      </c>
+      <c r="B104" s="20" t="s">
         <v>240</v>
       </c>
-    </row>
-    <row r="103" spans="1:5" x14ac:dyDescent="0.4">
-      <c r="A103" s="21" t="s">
-        <v>191</v>
-      </c>
-      <c r="B103" s="20" t="s">
+      <c r="C104" s="20" t="s">
+        <v>240</v>
+      </c>
+      <c r="D104" s="21" t="s">
         <v>241</v>
       </c>
-      <c r="C103" s="20" t="s">
-        <v>241</v>
-      </c>
-      <c r="D103" s="21" t="s">
-        <v>242</v>
-      </c>
-      <c r="E103" s="21"/>
-    </row>
-    <row r="104" spans="1:5" x14ac:dyDescent="0.4">
-      <c r="A104" s="15" t="s">
-        <v>243</v>
-      </c>
-      <c r="B104" s="18" t="s">
-        <v>244</v>
-      </c>
-      <c r="C104" s="18" t="s">
-        <v>244</v>
-      </c>
-      <c r="D104" s="15" t="s">
-        <v>245</v>
-      </c>
+      <c r="E104" s="21"/>
     </row>
     <row r="105" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A105" s="15" t="s">
+        <v>242</v>
+      </c>
+      <c r="B105" s="18" t="s">
         <v>243</v>
       </c>
-      <c r="B105" s="18" t="s">
-        <v>246</v>
-      </c>
       <c r="C105" s="18" t="s">
-        <v>246</v>
+        <v>243</v>
       </c>
       <c r="D105" s="15" t="s">
-        <v>247</v>
+        <v>244</v>
       </c>
     </row>
     <row r="106" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A106" s="15" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="B106" s="18" t="s">
-        <v>248</v>
+        <v>245</v>
       </c>
       <c r="C106" s="18" t="s">
-        <v>248</v>
+        <v>245</v>
       </c>
       <c r="D106" s="15" t="s">
-        <v>249</v>
+        <v>246</v>
       </c>
     </row>
     <row r="107" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A107" s="15" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="B107" s="18" t="s">
-        <v>250</v>
+        <v>247</v>
       </c>
       <c r="C107" s="18" t="s">
-        <v>250</v>
+        <v>247</v>
       </c>
       <c r="D107" s="15" t="s">
-        <v>251</v>
+        <v>248</v>
       </c>
     </row>
     <row r="108" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A108" s="15" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="B108" s="18" t="s">
-        <v>252</v>
+        <v>249</v>
       </c>
       <c r="C108" s="18" t="s">
-        <v>252</v>
+        <v>249</v>
       </c>
       <c r="D108" s="15" t="s">
-        <v>253</v>
+        <v>250</v>
       </c>
     </row>
     <row r="109" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A109" s="15" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="B109" s="18" t="s">
-        <v>254</v>
+        <v>251</v>
       </c>
       <c r="C109" s="18" t="s">
-        <v>254</v>
+        <v>251</v>
       </c>
       <c r="D109" s="15" t="s">
-        <v>255</v>
+        <v>252</v>
       </c>
     </row>
     <row r="110" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A110" s="15" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="B110" s="18" t="s">
-        <v>256</v>
+        <v>253</v>
       </c>
       <c r="C110" s="18" t="s">
-        <v>256</v>
+        <v>253</v>
       </c>
       <c r="D110" s="15" t="s">
-        <v>257</v>
+        <v>254</v>
       </c>
     </row>
     <row r="111" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A111" s="15" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="B111" s="18" t="s">
-        <v>258</v>
+        <v>255</v>
       </c>
       <c r="C111" s="18" t="s">
-        <v>258</v>
+        <v>255</v>
       </c>
       <c r="D111" s="15" t="s">
-        <v>259</v>
+        <v>256</v>
       </c>
     </row>
     <row r="112" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A112" s="15" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="B112" s="18" t="s">
-        <v>260</v>
+        <v>257</v>
       </c>
       <c r="C112" s="18" t="s">
-        <v>260</v>
+        <v>257</v>
       </c>
       <c r="D112" s="15" t="s">
-        <v>261</v>
+        <v>258</v>
       </c>
     </row>
     <row r="113" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A113" s="15" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="B113" s="18" t="s">
-        <v>262</v>
+        <v>259</v>
       </c>
       <c r="C113" s="18" t="s">
-        <v>262</v>
+        <v>259</v>
       </c>
       <c r="D113" s="15" t="s">
-        <v>263</v>
+        <v>260</v>
       </c>
     </row>
     <row r="114" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A114" s="15" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="B114" s="18" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
       <c r="C114" s="18" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
       <c r="D114" s="15" t="s">
-        <v>265</v>
+        <v>262</v>
       </c>
     </row>
     <row r="115" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A115" s="15" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="B115" s="18" t="s">
-        <v>266</v>
+        <v>263</v>
       </c>
       <c r="C115" s="18" t="s">
-        <v>266</v>
+        <v>263</v>
       </c>
       <c r="D115" s="15" t="s">
-        <v>267</v>
+        <v>264</v>
       </c>
     </row>
     <row r="116" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A116" s="15" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="B116" s="18" t="s">
-        <v>268</v>
+        <v>265</v>
       </c>
       <c r="C116" s="18" t="s">
-        <v>268</v>
+        <v>265</v>
       </c>
       <c r="D116" s="15" t="s">
-        <v>269</v>
+        <v>266</v>
       </c>
     </row>
     <row r="117" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A117" s="15" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="B117" s="18" t="s">
-        <v>270</v>
+        <v>267</v>
       </c>
       <c r="C117" s="18" t="s">
-        <v>270</v>
+        <v>267</v>
       </c>
       <c r="D117" s="15" t="s">
-        <v>271</v>
+        <v>268</v>
       </c>
     </row>
     <row r="118" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A118" s="15" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="B118" s="18" t="s">
-        <v>272</v>
+        <v>269</v>
       </c>
       <c r="C118" s="18" t="s">
-        <v>272</v>
+        <v>269</v>
       </c>
       <c r="D118" s="15" t="s">
-        <v>273</v>
+        <v>270</v>
       </c>
     </row>
     <row r="119" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A119" s="15" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="B119" s="18" t="s">
-        <v>274</v>
+        <v>271</v>
       </c>
       <c r="C119" s="18" t="s">
-        <v>274</v>
+        <v>271</v>
       </c>
       <c r="D119" s="15" t="s">
-        <v>275</v>
+        <v>272</v>
       </c>
     </row>
     <row r="120" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A120" s="15" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="B120" s="18" t="s">
-        <v>276</v>
+        <v>273</v>
       </c>
       <c r="C120" s="18" t="s">
-        <v>276</v>
+        <v>273</v>
       </c>
       <c r="D120" s="15" t="s">
-        <v>277</v>
+        <v>274</v>
       </c>
     </row>
     <row r="121" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A121" s="15" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="B121" s="18" t="s">
-        <v>278</v>
+        <v>275</v>
       </c>
       <c r="C121" s="18" t="s">
-        <v>278</v>
+        <v>275</v>
       </c>
       <c r="D121" s="15" t="s">
-        <v>279</v>
+        <v>276</v>
       </c>
     </row>
     <row r="122" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A122" s="15" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="B122" s="18" t="s">
-        <v>280</v>
+        <v>277</v>
       </c>
       <c r="C122" s="18" t="s">
-        <v>280</v>
+        <v>277</v>
       </c>
       <c r="D122" s="15" t="s">
-        <v>281</v>
+        <v>278</v>
       </c>
     </row>
     <row r="123" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A123" s="15" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="B123" s="18" t="s">
-        <v>282</v>
+        <v>279</v>
       </c>
       <c r="C123" s="18" t="s">
-        <v>282</v>
+        <v>279</v>
       </c>
       <c r="D123" s="15" t="s">
-        <v>283</v>
+        <v>280</v>
       </c>
     </row>
     <row r="124" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A124" s="15" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="B124" s="18" t="s">
-        <v>284</v>
+        <v>281</v>
       </c>
       <c r="C124" s="18" t="s">
-        <v>284</v>
+        <v>281</v>
       </c>
       <c r="D124" s="15" t="s">
-        <v>285</v>
+        <v>282</v>
       </c>
     </row>
     <row r="125" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A125" s="15" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="B125" s="18" t="s">
-        <v>286</v>
+        <v>283</v>
       </c>
       <c r="C125" s="18" t="s">
-        <v>286</v>
+        <v>283</v>
       </c>
       <c r="D125" s="15" t="s">
-        <v>287</v>
+        <v>284</v>
       </c>
     </row>
     <row r="126" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A126" s="15" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="B126" s="18" t="s">
-        <v>288</v>
+        <v>285</v>
       </c>
       <c r="C126" s="18" t="s">
-        <v>288</v>
+        <v>285</v>
       </c>
       <c r="D126" s="15" t="s">
-        <v>289</v>
+        <v>286</v>
       </c>
     </row>
     <row r="127" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A127" s="15" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="B127" s="18" t="s">
-        <v>290</v>
+        <v>287</v>
       </c>
       <c r="C127" s="18" t="s">
-        <v>290</v>
+        <v>287</v>
       </c>
       <c r="D127" s="15" t="s">
-        <v>291</v>
+        <v>288</v>
       </c>
     </row>
     <row r="128" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A128" s="15" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="B128" s="18" t="s">
-        <v>292</v>
+        <v>289</v>
       </c>
       <c r="C128" s="18" t="s">
-        <v>292</v>
+        <v>289</v>
       </c>
       <c r="D128" s="15" t="s">
-        <v>293</v>
+        <v>290</v>
       </c>
     </row>
     <row r="129" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A129" s="15" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="B129" s="18" t="s">
-        <v>294</v>
+        <v>291</v>
       </c>
       <c r="C129" s="18" t="s">
-        <v>294</v>
+        <v>291</v>
       </c>
       <c r="D129" s="15" t="s">
-        <v>295</v>
+        <v>292</v>
       </c>
     </row>
     <row r="130" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A130" s="15" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="B130" s="18" t="s">
-        <v>296</v>
+        <v>293</v>
       </c>
       <c r="C130" s="18" t="s">
-        <v>296</v>
+        <v>293</v>
       </c>
       <c r="D130" s="15" t="s">
-        <v>297</v>
+        <v>294</v>
       </c>
     </row>
     <row r="131" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A131" s="15" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="B131" s="18" t="s">
-        <v>298</v>
+        <v>295</v>
       </c>
       <c r="C131" s="18" t="s">
-        <v>298</v>
+        <v>295</v>
       </c>
       <c r="D131" s="15" t="s">
-        <v>299</v>
+        <v>296</v>
       </c>
     </row>
     <row r="132" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A132" s="15" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="B132" s="18" t="s">
-        <v>300</v>
+        <v>297</v>
       </c>
       <c r="C132" s="18" t="s">
-        <v>300</v>
+        <v>297</v>
       </c>
       <c r="D132" s="15" t="s">
-        <v>301</v>
+        <v>298</v>
       </c>
     </row>
     <row r="133" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A133" s="15" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="B133" s="18" t="s">
-        <v>302</v>
+        <v>299</v>
       </c>
       <c r="C133" s="18" t="s">
-        <v>302</v>
+        <v>299</v>
       </c>
       <c r="D133" s="15" t="s">
-        <v>303</v>
+        <v>300</v>
       </c>
     </row>
     <row r="134" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A134" s="15" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="B134" s="18" t="s">
-        <v>304</v>
+        <v>301</v>
       </c>
       <c r="C134" s="18" t="s">
-        <v>304</v>
+        <v>301</v>
       </c>
       <c r="D134" s="15" t="s">
-        <v>305</v>
+        <v>302</v>
       </c>
     </row>
     <row r="135" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A135" s="15" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="B135" s="18" t="s">
-        <v>306</v>
+        <v>303</v>
       </c>
       <c r="C135" s="18" t="s">
-        <v>306</v>
+        <v>303</v>
       </c>
       <c r="D135" s="15" t="s">
-        <v>307</v>
+        <v>304</v>
       </c>
     </row>
     <row r="136" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A136" s="15" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="B136" s="18" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="C136" s="18" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="D136" s="15" t="s">
-        <v>309</v>
+        <v>306</v>
       </c>
     </row>
     <row r="137" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A137" s="15" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="B137" s="18" t="s">
-        <v>310</v>
+        <v>307</v>
       </c>
       <c r="C137" s="18" t="s">
-        <v>310</v>
+        <v>307</v>
       </c>
       <c r="D137" s="15" t="s">
-        <v>311</v>
+        <v>308</v>
       </c>
     </row>
     <row r="138" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A138" s="15" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="B138" s="18" t="s">
-        <v>312</v>
+        <v>309</v>
       </c>
       <c r="C138" s="18" t="s">
-        <v>312</v>
+        <v>309</v>
       </c>
       <c r="D138" s="15" t="s">
-        <v>313</v>
+        <v>310</v>
       </c>
     </row>
     <row r="139" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A139" s="15" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="B139" s="18" t="s">
-        <v>314</v>
+        <v>311</v>
       </c>
       <c r="C139" s="18" t="s">
-        <v>314</v>
+        <v>311</v>
       </c>
       <c r="D139" s="15" t="s">
-        <v>315</v>
+        <v>312</v>
       </c>
     </row>
     <row r="140" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A140" s="15" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="B140" s="18" t="s">
-        <v>316</v>
+        <v>313</v>
       </c>
       <c r="C140" s="18" t="s">
-        <v>316</v>
+        <v>313</v>
       </c>
       <c r="D140" s="15" t="s">
-        <v>317</v>
+        <v>314</v>
       </c>
     </row>
     <row r="141" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A141" s="15" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="B141" s="18" t="s">
-        <v>318</v>
+        <v>315</v>
       </c>
       <c r="C141" s="18" t="s">
-        <v>318</v>
+        <v>315</v>
       </c>
       <c r="D141" s="15" t="s">
-        <v>319</v>
+        <v>316</v>
       </c>
     </row>
     <row r="142" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A142" s="15" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="B142" s="18" t="s">
-        <v>320</v>
+        <v>317</v>
       </c>
       <c r="C142" s="18" t="s">
-        <v>320</v>
+        <v>317</v>
       </c>
       <c r="D142" s="15" t="s">
-        <v>321</v>
+        <v>318</v>
       </c>
     </row>
     <row r="143" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A143" s="15" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="B143" s="18" t="s">
-        <v>322</v>
+        <v>319</v>
       </c>
       <c r="C143" s="18" t="s">
-        <v>322</v>
+        <v>319</v>
       </c>
       <c r="D143" s="15" t="s">
-        <v>323</v>
+        <v>320</v>
       </c>
     </row>
     <row r="144" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A144" s="15" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="B144" s="18" t="s">
-        <v>324</v>
+        <v>321</v>
       </c>
       <c r="C144" s="18" t="s">
-        <v>324</v>
+        <v>321</v>
       </c>
       <c r="D144" s="15" t="s">
-        <v>325</v>
+        <v>322</v>
       </c>
     </row>
     <row r="145" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A145" s="15" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="B145" s="18" t="s">
-        <v>326</v>
+        <v>323</v>
       </c>
       <c r="C145" s="18" t="s">
-        <v>326</v>
+        <v>323</v>
       </c>
       <c r="D145" s="15" t="s">
-        <v>327</v>
+        <v>324</v>
       </c>
     </row>
     <row r="146" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A146" s="15" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="B146" s="18" t="s">
-        <v>328</v>
+        <v>325</v>
       </c>
       <c r="C146" s="18" t="s">
-        <v>328</v>
+        <v>325</v>
       </c>
       <c r="D146" s="15" t="s">
-        <v>329</v>
+        <v>326</v>
       </c>
     </row>
     <row r="147" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A147" s="15" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="B147" s="18" t="s">
-        <v>330</v>
+        <v>327</v>
       </c>
       <c r="C147" s="18" t="s">
-        <v>330</v>
+        <v>327</v>
       </c>
       <c r="D147" s="15" t="s">
-        <v>331</v>
+        <v>328</v>
       </c>
     </row>
     <row r="148" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A148" s="15" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="B148" s="18" t="s">
-        <v>332</v>
+        <v>329</v>
       </c>
       <c r="C148" s="18" t="s">
-        <v>332</v>
+        <v>329</v>
       </c>
       <c r="D148" s="15" t="s">
-        <v>333</v>
+        <v>330</v>
       </c>
     </row>
     <row r="149" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A149" s="15" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="B149" s="18" t="s">
+        <v>331</v>
+      </c>
+      <c r="C149" s="18" t="s">
+        <v>331</v>
+      </c>
+      <c r="D149" s="15" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="150" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A150" s="15" t="s">
+        <v>242</v>
+      </c>
+      <c r="B150" s="18" t="s">
+        <v>333</v>
+      </c>
+      <c r="C150" s="18" t="s">
+        <v>333</v>
+      </c>
+      <c r="D150" s="15" t="s">
         <v>334</v>
       </c>
-      <c r="C149" s="18" t="s">
-        <v>334</v>
-      </c>
-      <c r="D149" s="15" t="s">
+    </row>
+    <row r="151" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A151" s="21" t="s">
+        <v>242</v>
+      </c>
+      <c r="B151" s="20" t="s">
         <v>335</v>
       </c>
-    </row>
-    <row r="150" spans="1:5" x14ac:dyDescent="0.4">
-      <c r="A150" s="21" t="s">
-        <v>243</v>
-      </c>
-      <c r="B150" s="20" t="s">
+      <c r="C151" s="20" t="s">
+        <v>335</v>
+      </c>
+      <c r="D151" s="21" t="s">
         <v>336</v>
       </c>
-      <c r="C150" s="20" t="s">
-        <v>336</v>
-      </c>
-      <c r="D150" s="21" t="s">
-        <v>337</v>
-      </c>
-      <c r="E150" s="21"/>
-    </row>
-    <row r="151" spans="1:5" x14ac:dyDescent="0.4">
-      <c r="A151" s="15" t="s">
-        <v>377</v>
-      </c>
-      <c r="B151" s="18" t="s">
-        <v>378</v>
-      </c>
-      <c r="C151" s="18" t="s">
-        <v>380</v>
-      </c>
-      <c r="D151" s="15">
-        <v>1</v>
-      </c>
+      <c r="E151" s="21"/>
     </row>
     <row r="152" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A152" s="15" t="s">
+        <v>376</v>
+      </c>
+      <c r="B152" s="18" t="s">
         <v>377</v>
       </c>
-      <c r="B152" s="18" t="s">
+      <c r="C152" s="18" t="s">
         <v>379</v>
       </c>
-      <c r="C152" s="18" t="s">
-        <v>381</v>
-      </c>
       <c r="D152" s="15">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="153" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A153" s="15" t="s">
+        <v>376</v>
+      </c>
+      <c r="B153" s="18" t="s">
+        <v>378</v>
+      </c>
+      <c r="C153" s="18" t="s">
+        <v>380</v>
+      </c>
+      <c r="D153" s="15">
         <v>0</v>
       </c>
     </row>
@@ -4781,26 +4823,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="7ab8c0d4-f18b-4fef-b649-c77d178c2495">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="65efab6e-20b9-465e-9733-f0c2ab732419" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x0101003456B0730C78B347BD7589BC061D6E7A" ma:contentTypeVersion="12" ma:contentTypeDescription="Crear nuevo documento." ma:contentTypeScope="" ma:versionID="63fa1c64418ad5e2c432e8a28af753ff">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="7ab8c0d4-f18b-4fef-b649-c77d178c2495" xmlns:ns3="65efab6e-20b9-465e-9733-f0c2ab732419" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="0084d3678d80c20d937c1596fa80271a" ns2:_="" ns3:_="">
     <xsd:import namespace="7ab8c0d4-f18b-4fef-b649-c77d178c2495"/>
@@ -5001,10 +5023,41 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="7ab8c0d4-f18b-4fef-b649-c77d178c2495">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="65efab6e-20b9-465e-9733-f0c2ab732419" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6F679A37-EAB5-400F-BBD1-820A1C585485}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{15651A92-013D-43FC-A841-092862588564}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="7ab8c0d4-f18b-4fef-b649-c77d178c2495"/>
+    <ds:schemaRef ds:uri="65efab6e-20b9-465e-9733-f0c2ab732419"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -5027,20 +5080,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{15651A92-013D-43FC-A841-092862588564}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6F679A37-EAB5-400F-BBD1-820A1C585485}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="7ab8c0d4-f18b-4fef-b649-c77d178c2495"/>
-    <ds:schemaRef ds:uri="65efab6e-20b9-465e-9733-f0c2ab732419"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>